<commit_message>
Remove hardcoding of TRAJ_FAIL conditions
- Create a timeout duration value in adjustableSettings.cpp instead of hardcoding 2000 ms value in trajectory.cpp
- Update associated .h, .cpp files
- Update MATLAB-based settings parsing
</commit_message>
<xml_diff>
--- a/controller/tuning data/tuning data overview.xlsx
+++ b/controller/tuning data/tuning data overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cfolinus/Documents/MIT/CMF FIDL/07 Control/soft-actuator-controller/controller/tuning data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501E8234-46D7-FF47-8BE7-66F50D4D2250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9EA23EB-62B0-FE47-9860-A1E3D5C5D9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="780" windowWidth="34560" windowHeight="20640" activeTab="1" xr2:uid="{CB76BD02-C45A-F243-9B85-AA0FA8F12FFA}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34560" windowHeight="20640" activeTab="1" xr2:uid="{CB76BD02-C45A-F243-9B85-AA0FA8F12FFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Calibration files" sheetId="1" r:id="rId1"/>
@@ -309,9 +309,6 @@
     <t>Recommended default from Evan: 30 (ms)</t>
   </si>
   <si>
-    <t>THRESHOLD &gt; TRAJ_FAIL_PRESSURE</t>
-  </si>
-  <si>
     <t>TRAJ_FAIL_TIME</t>
   </si>
   <si>
@@ -325,6 +322,9 @@
   </si>
   <si>
     <t>Test specific</t>
+  </si>
+  <si>
+    <t>TRAJ_FAIL_PRESSURE</t>
   </si>
 </sst>
 </file>
@@ -942,7 +942,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -991,18 +991,6 @@
     <xf numFmtId="9" fontId="1" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="19" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1011,43 +999,18 @@
     <xf numFmtId="0" fontId="3" fillId="18" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="22" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1100,6 +1063,57 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="23" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="23" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2733,469 +2747,466 @@
   <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" style="59" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" style="59" customWidth="1"/>
-    <col min="3" max="3" width="48.42578125" customWidth="1"/>
-    <col min="4" max="5" width="45.7109375" customWidth="1"/>
-    <col min="6" max="6" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="5.7109375" style="44" customWidth="1"/>
+    <col min="3" max="6" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1" thickBot="1">
-      <c r="A1" s="60"/>
-      <c r="B1" s="38" t="s">
+      <c r="A1" s="45"/>
+      <c r="B1" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="39"/>
-      <c r="D1" s="40" t="s">
+      <c r="C1" s="33"/>
+      <c r="D1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="41" t="s">
+      <c r="E1" s="73" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="20" customHeight="1">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="58" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="37" t="s">
+      <c r="E2" s="59" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="20" customHeight="1">
-      <c r="A3" s="62"/>
+      <c r="A3" s="47"/>
       <c r="B3" s="21"/>
       <c r="C3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="30">
+      <c r="D3" s="60">
         <v>0.06</v>
       </c>
-      <c r="E3" s="28">
+      <c r="E3" s="61">
         <v>-0.122</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="20" customHeight="1">
-      <c r="A4" s="62"/>
+      <c r="A4" s="47"/>
       <c r="B4" s="21"/>
       <c r="C4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="30">
+      <c r="D4" s="60">
         <v>151</v>
       </c>
-      <c r="E4" s="28">
+      <c r="E4" s="61">
         <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="20" customHeight="1">
-      <c r="A5" s="62"/>
+      <c r="A5" s="47"/>
       <c r="B5" s="21"/>
       <c r="C5" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="60">
         <v>183</v>
       </c>
-      <c r="E5" s="28">
+      <c r="E5" s="61">
         <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="20" customHeight="1">
-      <c r="A6" s="62"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="21"/>
       <c r="C6" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="30">
+      <c r="D6" s="60">
         <v>0.11</v>
       </c>
-      <c r="E6" s="28">
+      <c r="E6" s="61">
         <v>0.11</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="20" customHeight="1">
-      <c r="A7" s="62"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="21"/>
       <c r="C7" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="60">
         <f>D3-D6</f>
         <v>-0.05</v>
       </c>
-      <c r="E7" s="28">
+      <c r="E7" s="61">
         <f>E3-E6</f>
         <v>-0.23199999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="20" customHeight="1">
-      <c r="A8" s="62"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="22" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="31" t="s">
+      <c r="D8" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="63" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="20" customHeight="1">
-      <c r="A9" s="62"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="22"/>
       <c r="C9" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="30">
+      <c r="D9" s="60">
         <v>0.06</v>
       </c>
-      <c r="E9" s="28">
+      <c r="E9" s="61">
         <v>-0.122</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="20" customHeight="1">
-      <c r="A10" s="62"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="22"/>
       <c r="C10" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="30">
+      <c r="D10" s="60">
         <v>145</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="61">
         <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="20" customHeight="1">
-      <c r="A11" s="62"/>
+      <c r="A11" s="47"/>
       <c r="B11" s="22"/>
       <c r="C11" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="30">
+      <c r="D11" s="60">
         <v>158</v>
       </c>
-      <c r="E11" s="28">
+      <c r="E11" s="61">
         <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="20" customHeight="1">
-      <c r="A12" s="62"/>
+      <c r="A12" s="47"/>
       <c r="B12" s="22"/>
       <c r="C12" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="30">
+      <c r="D12" s="60">
         <v>0.11</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="61">
         <v>0.11</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="20" customHeight="1" thickBot="1">
-      <c r="A13" s="63"/>
-      <c r="B13" s="42"/>
-      <c r="C13" s="43" t="s">
+      <c r="A13" s="48"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="D13" s="44">
+      <c r="D13" s="64">
         <f>D9-D12</f>
         <v>-0.05</v>
       </c>
-      <c r="E13" s="45">
+      <c r="E13" s="65">
         <f>E9-E12</f>
         <v>-0.23199999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="20" customHeight="1" thickBot="1">
-      <c r="A14" s="64"/>
-      <c r="B14" s="56"/>
+      <c r="A14" s="49"/>
+      <c r="B14" s="41"/>
       <c r="C14" s="23"/>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="E14" s="47" t="s">
-        <v>1</v>
-      </c>
-      <c r="F14" s="52" t="s">
+      <c r="E14" s="74" t="s">
+        <v>1</v>
+      </c>
+      <c r="F14" s="37" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="20" customHeight="1">
-      <c r="A15" s="65" t="s">
+      <c r="A15" s="50" t="s">
+        <v>86</v>
+      </c>
+      <c r="B15" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="57" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="68" t="s">
+      <c r="C15" s="53" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="46">
+      <c r="D15" s="66">
         <f>D4</f>
         <v>151</v>
       </c>
-      <c r="E15" s="48">
+      <c r="E15" s="67">
         <f>E4</f>
         <v>145</v>
       </c>
-      <c r="F15" s="51"/>
+      <c r="F15" s="36"/>
     </row>
     <row r="16" spans="1:6" ht="20" customHeight="1">
-      <c r="A16" s="66"/>
-      <c r="B16" s="58"/>
-      <c r="C16" s="69" t="s">
+      <c r="A16" s="51"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="32">
+      <c r="D16" s="68">
         <f>D5</f>
         <v>183</v>
       </c>
-      <c r="E16" s="49">
+      <c r="E16" s="69">
         <f>E5</f>
         <v>173</v>
       </c>
-      <c r="F16" s="32"/>
+      <c r="F16" s="28"/>
     </row>
     <row r="17" spans="1:6" ht="20" customHeight="1">
-      <c r="A17" s="66"/>
-      <c r="B17" s="58"/>
-      <c r="C17" s="69" t="s">
+      <c r="A17" s="51"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="54" t="s">
         <v>69</v>
       </c>
-      <c r="D17" s="32">
+      <c r="D17" s="68">
         <f>D10</f>
         <v>145</v>
       </c>
-      <c r="E17" s="49">
+      <c r="E17" s="69">
         <f>E10</f>
         <v>143</v>
       </c>
-      <c r="F17" s="32"/>
+      <c r="F17" s="28"/>
     </row>
     <row r="18" spans="1:6" ht="20" customHeight="1">
-      <c r="A18" s="66"/>
-      <c r="B18" s="58"/>
-      <c r="C18" s="69" t="s">
+      <c r="A18" s="51"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="54" t="s">
         <v>70</v>
       </c>
-      <c r="D18" s="32">
+      <c r="D18" s="68">
         <f>D11</f>
         <v>158</v>
       </c>
-      <c r="E18" s="49">
+      <c r="E18" s="69">
         <f>E11</f>
         <v>169</v>
       </c>
-      <c r="F18" s="32"/>
+      <c r="F18" s="28"/>
     </row>
     <row r="19" spans="1:6" ht="20" customHeight="1">
-      <c r="A19" s="66"/>
-      <c r="B19" s="58"/>
-      <c r="C19" s="69" t="s">
+      <c r="A19" s="51"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="54" t="s">
         <v>73</v>
       </c>
-      <c r="D19" s="32">
+      <c r="D19" s="68">
         <f>D7</f>
         <v>-0.05</v>
       </c>
-      <c r="E19" s="49">
+      <c r="E19" s="69">
         <f>E7</f>
         <v>-0.23199999999999998</v>
       </c>
-      <c r="F19" s="32"/>
+      <c r="F19" s="28"/>
     </row>
     <row r="20" spans="1:6" ht="20" customHeight="1">
-      <c r="A20" s="66"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="20"/>
-      <c r="C20" s="70"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="32"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="28"/>
     </row>
     <row r="21" spans="1:6" ht="20" customHeight="1">
-      <c r="A21" s="66"/>
-      <c r="B21" s="53" t="s">
+      <c r="A21" s="51"/>
+      <c r="B21" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="56" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" s="68"/>
+      <c r="E21" s="69"/>
+      <c r="F21" s="28" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="20" customHeight="1">
+      <c r="A22" s="51"/>
+      <c r="B22" s="39"/>
+      <c r="C22" s="56" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" s="68">
+        <v>0</v>
+      </c>
+      <c r="E22" s="69">
+        <v>0</v>
+      </c>
+      <c r="F22" s="28"/>
+    </row>
+    <row r="23" spans="1:6" ht="20" customHeight="1">
+      <c r="A23" s="51"/>
+      <c r="B23" s="39"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="68"/>
+      <c r="E23" s="69"/>
+      <c r="F23" s="28"/>
+    </row>
+    <row r="24" spans="1:6" ht="20" customHeight="1">
+      <c r="A24" s="51"/>
+      <c r="B24" s="39"/>
+      <c r="C24" s="56" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="68">
+        <v>30</v>
+      </c>
+      <c r="E24" s="69">
+        <v>30</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="20" customHeight="1">
+      <c r="A25" s="51"/>
+      <c r="B25" s="39"/>
+      <c r="C25" s="56" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25" s="68">
+        <v>30</v>
+      </c>
+      <c r="E25" s="69">
+        <v>30</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="20" customHeight="1">
+      <c r="A26" s="51"/>
+      <c r="B26" s="39"/>
+      <c r="C26" s="56" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" s="68">
+        <v>30</v>
+      </c>
+      <c r="E26" s="69">
+        <v>30</v>
+      </c>
+      <c r="F26" s="28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="20" customHeight="1">
+      <c r="A27" s="51"/>
+      <c r="B27" s="39"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="68"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="28"/>
+    </row>
+    <row r="28" spans="1:6" ht="20" customHeight="1">
+      <c r="A28" s="51"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="71" t="s">
-        <v>71</v>
-      </c>
-      <c r="D21" s="32"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="32" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="20" customHeight="1">
-      <c r="A22" s="66"/>
-      <c r="B22" s="54"/>
-      <c r="C22" s="71" t="s">
-        <v>72</v>
-      </c>
-      <c r="D22" s="32">
-        <v>0</v>
-      </c>
-      <c r="E22" s="49">
-        <v>0</v>
-      </c>
-      <c r="F22" s="32"/>
-    </row>
-    <row r="23" spans="1:6" ht="20" customHeight="1">
-      <c r="A23" s="66"/>
-      <c r="B23" s="54"/>
-      <c r="C23" s="70"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="32"/>
-    </row>
-    <row r="24" spans="1:6" ht="20" customHeight="1">
-      <c r="A24" s="66"/>
-      <c r="B24" s="54"/>
-      <c r="C24" s="71" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="32">
-        <v>30</v>
-      </c>
-      <c r="E24" s="49">
-        <v>30</v>
-      </c>
-      <c r="F24" s="32" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="20" customHeight="1">
-      <c r="A25" s="66"/>
-      <c r="B25" s="54"/>
-      <c r="C25" s="71" t="s">
-        <v>75</v>
-      </c>
-      <c r="D25" s="32">
-        <v>30</v>
-      </c>
-      <c r="E25" s="49">
-        <v>30</v>
-      </c>
-      <c r="F25" s="32" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="20" customHeight="1">
-      <c r="A26" s="66"/>
-      <c r="B26" s="54"/>
-      <c r="C26" s="71" t="s">
-        <v>76</v>
-      </c>
-      <c r="D26" s="32">
-        <v>30</v>
-      </c>
-      <c r="E26" s="49">
-        <v>30</v>
-      </c>
-      <c r="F26" s="32" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="20" customHeight="1">
-      <c r="A27" s="66"/>
-      <c r="B27" s="54"/>
-      <c r="C27" s="70"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="32"/>
-    </row>
-    <row r="28" spans="1:6" ht="20" customHeight="1">
-      <c r="A28" s="66"/>
-      <c r="B28" s="54"/>
-      <c r="C28" s="71" t="s">
+      <c r="D28" s="68"/>
+      <c r="E28" s="69"/>
+      <c r="F28" s="28"/>
+    </row>
+    <row r="29" spans="1:6" ht="20" customHeight="1">
+      <c r="A29" s="51"/>
+      <c r="B29" s="39"/>
+      <c r="C29" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="D28" s="32"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="32"/>
-    </row>
-    <row r="29" spans="1:6" ht="20" customHeight="1">
-      <c r="A29" s="66"/>
-      <c r="B29" s="54"/>
-      <c r="C29" s="71" t="s">
+      <c r="D29" s="68"/>
+      <c r="E29" s="69"/>
+      <c r="F29" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="D29" s="32"/>
-      <c r="E29" s="49"/>
-      <c r="F29" s="32" t="s">
-        <v>86</v>
-      </c>
     </row>
     <row r="30" spans="1:6" ht="20" customHeight="1">
-      <c r="A30" s="66"/>
-      <c r="B30" s="54"/>
-      <c r="C30" s="71" t="s">
+      <c r="A30" s="51"/>
+      <c r="B30" s="39"/>
+      <c r="C30" s="56" t="s">
         <v>77</v>
       </c>
-      <c r="D30" s="32"/>
-      <c r="E30" s="49"/>
-      <c r="F30" s="32"/>
+      <c r="D30" s="68"/>
+      <c r="E30" s="69"/>
+      <c r="F30" s="28"/>
     </row>
     <row r="31" spans="1:6" ht="20" customHeight="1">
-      <c r="A31" s="66"/>
-      <c r="B31" s="54"/>
-      <c r="C31" s="71" t="s">
+      <c r="A31" s="51"/>
+      <c r="B31" s="39"/>
+      <c r="C31" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="32"/>
-      <c r="E31" s="49"/>
-      <c r="F31" s="32"/>
+      <c r="D31" s="68"/>
+      <c r="E31" s="69"/>
+      <c r="F31" s="28"/>
     </row>
     <row r="32" spans="1:6" ht="20" customHeight="1">
-      <c r="A32" s="66"/>
-      <c r="B32" s="54"/>
-      <c r="C32" s="71" t="s">
+      <c r="A32" s="51"/>
+      <c r="B32" s="39"/>
+      <c r="C32" s="56" t="s">
         <v>79</v>
       </c>
-      <c r="D32" s="32"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="32"/>
+      <c r="D32" s="68"/>
+      <c r="E32" s="69"/>
+      <c r="F32" s="28"/>
     </row>
     <row r="33" spans="1:6" ht="20" customHeight="1">
-      <c r="A33" s="66"/>
-      <c r="B33" s="54"/>
-      <c r="C33" s="70"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="32"/>
+      <c r="A33" s="51"/>
+      <c r="B33" s="39"/>
+      <c r="C33" s="55"/>
+      <c r="D33" s="68"/>
+      <c r="E33" s="69"/>
+      <c r="F33" s="28"/>
     </row>
     <row r="34" spans="1:6" ht="20" customHeight="1">
-      <c r="A34" s="66"/>
-      <c r="B34" s="54"/>
-      <c r="C34" s="71" t="s">
+      <c r="A34" s="51"/>
+      <c r="B34" s="39"/>
+      <c r="C34" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="D34" s="32"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="32"/>
+      <c r="D34" s="68"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="28"/>
     </row>
     <row r="35" spans="1:6" ht="20" customHeight="1" thickBot="1">
-      <c r="A35" s="67"/>
-      <c r="B35" s="55"/>
-      <c r="C35" s="72" t="s">
+      <c r="A35" s="52"/>
+      <c r="B35" s="40"/>
+      <c r="C35" s="57" t="s">
         <v>81</v>
       </c>
-      <c r="D35" s="33"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="33"/>
+      <c r="D35" s="70"/>
+      <c r="E35" s="71"/>
+      <c r="F35" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Add ability to use custom adjustableSettings files
- To change adjustableSettings reference, add name of the adjustableSettings file ("adjustableSettings*.cpp") to the src_filter in platformio.ini
</commit_message>
<xml_diff>
--- a/controller/tuning data/tuning data overview.xlsx
+++ b/controller/tuning data/tuning data overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cfolinus/Documents/MIT/CMF FIDL/07 Control/soft-actuator-controller/controller/tuning data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9EA23EB-62B0-FE47-9860-A1E3D5C5D9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABACB3D-81B3-0544-8408-109F165D36AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34560" windowHeight="20640" activeTab="1" xr2:uid="{CB76BD02-C45A-F243-9B85-AA0FA8F12FFA}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="26360" windowHeight="20640" activeTab="1" xr2:uid="{CB76BD02-C45A-F243-9B85-AA0FA8F12FFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Calibration files" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="93">
   <si>
     <t>Kim Possible</t>
   </si>
@@ -325,6 +325,15 @@
   </si>
   <si>
     <t>TRAJ_FAIL_PRESSURE</t>
+  </si>
+  <si>
+    <t>adjustableSettings_kim</t>
+  </si>
+  <si>
+    <t>adjustableSettings_ron</t>
+  </si>
+  <si>
+    <t>Settings filename [.cpp]</t>
   </si>
 </sst>
 </file>
@@ -508,7 +517,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -577,10 +586,40 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -634,11 +673,13 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="medium">
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -702,21 +743,6 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -858,14 +884,16 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -874,6 +902,17 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -881,7 +920,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -892,47 +933,12 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -942,7 +948,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -972,6 +978,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
@@ -979,141 +988,148 @@
       <alignment horizontal="left" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="18" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="1" fillId="17" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90"/>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2744,7 +2760,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A87AAE91-719E-6140-A33F-D8F6685EEC6D}">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="2" width="5.7109375" style="44" customWidth="1"/>
@@ -2753,14 +2769,14 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1" thickBot="1">
       <c r="A1" s="45"/>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="72" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="73" t="s">
+      <c r="E1" s="59" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2768,453 +2784,475 @@
       <c r="A2" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="58" t="s">
+      <c r="D2" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="59" t="s">
+      <c r="E2" s="51" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="20" customHeight="1">
       <c r="A3" s="47"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="24" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="60">
+      <c r="D3" s="52">
         <v>0.06</v>
       </c>
-      <c r="E3" s="61">
+      <c r="E3" s="53">
         <v>-0.122</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="20" customHeight="1">
       <c r="A4" s="47"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="25" t="s">
+      <c r="B4" s="22"/>
+      <c r="C4" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="60">
+      <c r="D4" s="52">
         <v>151</v>
       </c>
-      <c r="E4" s="61">
+      <c r="E4" s="53">
         <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="20" customHeight="1">
       <c r="A5" s="47"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="25" t="s">
+      <c r="B5" s="22"/>
+      <c r="C5" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="60">
+      <c r="D5" s="52">
         <v>183</v>
       </c>
-      <c r="E5" s="61">
+      <c r="E5" s="53">
         <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="20" customHeight="1">
       <c r="A6" s="47"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="24" t="s">
+      <c r="B6" s="22"/>
+      <c r="C6" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="60">
+      <c r="D6" s="52">
         <v>0.11</v>
       </c>
-      <c r="E6" s="61">
+      <c r="E6" s="53">
         <v>0.11</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="20" customHeight="1">
       <c r="A7" s="47"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="24" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="60">
+      <c r="D7" s="52">
         <f>D3-D6</f>
         <v>-0.05</v>
       </c>
-      <c r="E7" s="61">
+      <c r="E7" s="53">
         <f>E3-E6</f>
         <v>-0.23199999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="20" customHeight="1">
       <c r="A8" s="47"/>
-      <c r="B8" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="26" t="s">
+      <c r="B8" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="62" t="s">
+      <c r="D8" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="63" t="s">
+      <c r="E8" s="55" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="20" customHeight="1">
       <c r="A9" s="47"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="26" t="s">
+      <c r="B9" s="23"/>
+      <c r="C9" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="60">
+      <c r="D9" s="52">
         <v>0.06</v>
       </c>
-      <c r="E9" s="61">
+      <c r="E9" s="53">
         <v>-0.122</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="20" customHeight="1">
       <c r="A10" s="47"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="27" t="s">
+      <c r="B10" s="23"/>
+      <c r="C10" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="60">
+      <c r="D10" s="52">
         <v>145</v>
       </c>
-      <c r="E10" s="61">
+      <c r="E10" s="53">
         <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="20" customHeight="1">
       <c r="A11" s="47"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="27" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="60">
+      <c r="D11" s="52">
         <v>158</v>
       </c>
-      <c r="E11" s="61">
+      <c r="E11" s="53">
         <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="20" customHeight="1">
       <c r="A12" s="47"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="26" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="60">
+      <c r="D12" s="52">
         <v>0.11</v>
       </c>
-      <c r="E12" s="61">
+      <c r="E12" s="53">
         <v>0.11</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="20" customHeight="1" thickBot="1">
       <c r="A13" s="48"/>
-      <c r="B13" s="34"/>
-      <c r="C13" s="35" t="s">
+      <c r="B13" s="35"/>
+      <c r="C13" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="D13" s="64">
+      <c r="D13" s="56">
         <f>D9-D12</f>
         <v>-0.05</v>
       </c>
-      <c r="E13" s="65">
+      <c r="E13" s="57">
         <f>E9-E12</f>
         <v>-0.23199999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="20" customHeight="1" thickBot="1">
       <c r="A14" s="49"/>
-      <c r="B14" s="41"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="72" t="s">
+      <c r="B14" s="42"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="E14" s="74" t="s">
-        <v>1</v>
-      </c>
-      <c r="F14" s="37" t="s">
+      <c r="E14" s="61" t="s">
+        <v>1</v>
+      </c>
+      <c r="F14" s="78" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="20" customHeight="1">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="64"/>
+      <c r="C15" s="66" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" s="69" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="65" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" s="66"/>
+    </row>
+    <row r="16" spans="1:6" ht="20" customHeight="1">
+      <c r="A16" s="38"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="73"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="67"/>
+    </row>
+    <row r="17" spans="1:6" ht="20" customHeight="1">
+      <c r="A17" s="38"/>
+      <c r="B17" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="53" t="s">
+      <c r="C17" s="74" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="66">
+      <c r="D17" s="71">
         <f>D4</f>
         <v>151</v>
       </c>
-      <c r="E15" s="67">
+      <c r="E17" s="40">
         <f>E4</f>
         <v>145</v>
       </c>
-      <c r="F15" s="36"/>
-    </row>
-    <row r="16" spans="1:6" ht="20" customHeight="1">
-      <c r="A16" s="51"/>
-      <c r="B16" s="43"/>
-      <c r="C16" s="54" t="s">
+      <c r="F17" s="25"/>
+    </row>
+    <row r="18" spans="1:6" ht="20" customHeight="1">
+      <c r="A18" s="38"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="74" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="68">
+      <c r="D18" s="71">
         <f>D5</f>
         <v>183</v>
       </c>
-      <c r="E16" s="69">
+      <c r="E18" s="40">
         <f>E5</f>
         <v>173</v>
       </c>
-      <c r="F16" s="28"/>
-    </row>
-    <row r="17" spans="1:6" ht="20" customHeight="1">
-      <c r="A17" s="51"/>
-      <c r="B17" s="43"/>
-      <c r="C17" s="54" t="s">
+      <c r="F18" s="25"/>
+    </row>
+    <row r="19" spans="1:6" ht="20" customHeight="1">
+      <c r="A19" s="38"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="74" t="s">
         <v>69</v>
       </c>
-      <c r="D17" s="68">
+      <c r="D19" s="71">
         <f>D10</f>
         <v>145</v>
       </c>
-      <c r="E17" s="69">
+      <c r="E19" s="40">
         <f>E10</f>
         <v>143</v>
       </c>
-      <c r="F17" s="28"/>
-    </row>
-    <row r="18" spans="1:6" ht="20" customHeight="1">
-      <c r="A18" s="51"/>
-      <c r="B18" s="43"/>
-      <c r="C18" s="54" t="s">
+      <c r="F19" s="25"/>
+    </row>
+    <row r="20" spans="1:6" ht="20" customHeight="1">
+      <c r="A20" s="38"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="74" t="s">
         <v>70</v>
       </c>
-      <c r="D18" s="68">
+      <c r="D20" s="71">
         <f>D11</f>
         <v>158</v>
       </c>
-      <c r="E18" s="69">
+      <c r="E20" s="40">
         <f>E11</f>
         <v>169</v>
       </c>
-      <c r="F18" s="28"/>
-    </row>
-    <row r="19" spans="1:6" ht="20" customHeight="1">
-      <c r="A19" s="51"/>
-      <c r="B19" s="43"/>
-      <c r="C19" s="54" t="s">
+      <c r="F20" s="25"/>
+    </row>
+    <row r="21" spans="1:6" ht="20" customHeight="1">
+      <c r="A21" s="38"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="D19" s="68">
+      <c r="D21" s="71">
         <f>D7</f>
         <v>-0.05</v>
       </c>
-      <c r="E19" s="69">
+      <c r="E21" s="40">
         <f>E7</f>
         <v>-0.23199999999999998</v>
       </c>
-      <c r="F19" s="28"/>
-    </row>
-    <row r="20" spans="1:6" ht="20" customHeight="1">
-      <c r="A20" s="51"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="55"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="69"/>
-      <c r="F20" s="28"/>
-    </row>
-    <row r="21" spans="1:6" ht="20" customHeight="1">
-      <c r="A21" s="51"/>
-      <c r="B21" s="38" t="s">
+      <c r="F21" s="25"/>
+    </row>
+    <row r="22" spans="1:6" ht="20" customHeight="1">
+      <c r="A22" s="38"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="75"/>
+      <c r="D22" s="71"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="25"/>
+    </row>
+    <row r="23" spans="1:6" ht="20" customHeight="1">
+      <c r="A23" s="38"/>
+      <c r="B23" s="63" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="56" t="s">
+      <c r="C23" s="76" t="s">
         <v>71</v>
       </c>
-      <c r="D21" s="68"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="28" t="s">
+      <c r="D23" s="71"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="25" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="20" customHeight="1">
-      <c r="A22" s="51"/>
-      <c r="B22" s="39"/>
-      <c r="C22" s="56" t="s">
+    <row r="24" spans="1:6" ht="20" customHeight="1">
+      <c r="A24" s="38"/>
+      <c r="B24" s="63"/>
+      <c r="C24" s="76" t="s">
         <v>72</v>
       </c>
-      <c r="D22" s="68">
+      <c r="D24" s="71">
         <v>0</v>
       </c>
-      <c r="E22" s="69">
+      <c r="E24" s="40">
         <v>0</v>
       </c>
-      <c r="F22" s="28"/>
-    </row>
-    <row r="23" spans="1:6" ht="20" customHeight="1">
-      <c r="A23" s="51"/>
-      <c r="B23" s="39"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="69"/>
-      <c r="F23" s="28"/>
-    </row>
-    <row r="24" spans="1:6" ht="20" customHeight="1">
-      <c r="A24" s="51"/>
-      <c r="B24" s="39"/>
-      <c r="C24" s="56" t="s">
+      <c r="F24" s="25"/>
+    </row>
+    <row r="25" spans="1:6" ht="20" customHeight="1">
+      <c r="A25" s="38"/>
+      <c r="B25" s="63"/>
+      <c r="C25" s="75"/>
+      <c r="D25" s="71"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="25"/>
+    </row>
+    <row r="26" spans="1:6" ht="20" customHeight="1">
+      <c r="A26" s="38"/>
+      <c r="B26" s="63"/>
+      <c r="C26" s="76" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="68">
+      <c r="D26" s="71">
         <v>30</v>
       </c>
-      <c r="E24" s="69">
+      <c r="E26" s="40">
         <v>30</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F26" s="25" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="20" customHeight="1">
-      <c r="A25" s="51"/>
-      <c r="B25" s="39"/>
-      <c r="C25" s="56" t="s">
+    <row r="27" spans="1:6" ht="20" customHeight="1">
+      <c r="A27" s="38"/>
+      <c r="B27" s="63"/>
+      <c r="C27" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="68">
+      <c r="D27" s="71">
         <v>30</v>
       </c>
-      <c r="E25" s="69">
+      <c r="E27" s="40">
         <v>30</v>
       </c>
-      <c r="F25" s="28" t="s">
+      <c r="F27" s="25" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="20" customHeight="1">
-      <c r="A26" s="51"/>
-      <c r="B26" s="39"/>
-      <c r="C26" s="56" t="s">
+    <row r="28" spans="1:6" ht="20" customHeight="1">
+      <c r="A28" s="38"/>
+      <c r="B28" s="63"/>
+      <c r="C28" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="D26" s="68">
+      <c r="D28" s="71">
         <v>30</v>
       </c>
-      <c r="E26" s="69">
+      <c r="E28" s="40">
         <v>30</v>
       </c>
-      <c r="F26" s="28" t="s">
+      <c r="F28" s="25" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="20" customHeight="1">
-      <c r="A27" s="51"/>
-      <c r="B27" s="39"/>
-      <c r="C27" s="55"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="69"/>
-      <c r="F27" s="28"/>
-    </row>
-    <row r="28" spans="1:6" ht="20" customHeight="1">
-      <c r="A28" s="51"/>
-      <c r="B28" s="39"/>
-      <c r="C28" s="56" t="s">
+    <row r="29" spans="1:6" ht="20" customHeight="1">
+      <c r="A29" s="38"/>
+      <c r="B29" s="63"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="71"/>
+      <c r="E29" s="40"/>
+      <c r="F29" s="25"/>
+    </row>
+    <row r="30" spans="1:6" ht="20" customHeight="1">
+      <c r="A30" s="38"/>
+      <c r="B30" s="63"/>
+      <c r="C30" s="76" t="s">
         <v>89</v>
       </c>
-      <c r="D28" s="68"/>
-      <c r="E28" s="69"/>
-      <c r="F28" s="28"/>
-    </row>
-    <row r="29" spans="1:6" ht="20" customHeight="1">
-      <c r="A29" s="51"/>
-      <c r="B29" s="39"/>
-      <c r="C29" s="56" t="s">
+      <c r="D30" s="71"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="25"/>
+    </row>
+    <row r="31" spans="1:6" ht="20" customHeight="1">
+      <c r="A31" s="38"/>
+      <c r="B31" s="63"/>
+      <c r="C31" s="76" t="s">
         <v>84</v>
       </c>
-      <c r="D29" s="68"/>
-      <c r="E29" s="69"/>
-      <c r="F29" s="28" t="s">
+      <c r="D31" s="71"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="25" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="20" customHeight="1">
-      <c r="A30" s="51"/>
-      <c r="B30" s="39"/>
-      <c r="C30" s="56" t="s">
+    <row r="32" spans="1:6" ht="20" customHeight="1">
+      <c r="A32" s="38"/>
+      <c r="B32" s="63"/>
+      <c r="C32" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="D30" s="68"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="28"/>
-    </row>
-    <row r="31" spans="1:6" ht="20" customHeight="1">
-      <c r="A31" s="51"/>
-      <c r="B31" s="39"/>
-      <c r="C31" s="56" t="s">
+      <c r="D32" s="71"/>
+      <c r="E32" s="40"/>
+      <c r="F32" s="25"/>
+    </row>
+    <row r="33" spans="1:6" ht="20" customHeight="1">
+      <c r="A33" s="38"/>
+      <c r="B33" s="63"/>
+      <c r="C33" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="68"/>
-      <c r="E31" s="69"/>
-      <c r="F31" s="28"/>
-    </row>
-    <row r="32" spans="1:6" ht="20" customHeight="1">
-      <c r="A32" s="51"/>
-      <c r="B32" s="39"/>
-      <c r="C32" s="56" t="s">
+      <c r="D33" s="71"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="25"/>
+    </row>
+    <row r="34" spans="1:6" ht="20" customHeight="1">
+      <c r="A34" s="38"/>
+      <c r="B34" s="63"/>
+      <c r="C34" s="76" t="s">
         <v>79</v>
       </c>
-      <c r="D32" s="68"/>
-      <c r="E32" s="69"/>
-      <c r="F32" s="28"/>
-    </row>
-    <row r="33" spans="1:6" ht="20" customHeight="1">
-      <c r="A33" s="51"/>
-      <c r="B33" s="39"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="68"/>
-      <c r="E33" s="69"/>
-      <c r="F33" s="28"/>
-    </row>
-    <row r="34" spans="1:6" ht="20" customHeight="1">
-      <c r="A34" s="51"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="56" t="s">
+      <c r="D34" s="71"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="25"/>
+    </row>
+    <row r="35" spans="1:6" ht="20" customHeight="1">
+      <c r="A35" s="38"/>
+      <c r="B35" s="63"/>
+      <c r="C35" s="75"/>
+      <c r="D35" s="71"/>
+      <c r="E35" s="40"/>
+      <c r="F35" s="25"/>
+    </row>
+    <row r="36" spans="1:6" ht="20" customHeight="1">
+      <c r="A36" s="38"/>
+      <c r="B36" s="63"/>
+      <c r="C36" s="76" t="s">
         <v>80</v>
       </c>
-      <c r="D34" s="68"/>
-      <c r="E34" s="69"/>
-      <c r="F34" s="28"/>
-    </row>
-    <row r="35" spans="1:6" ht="20" customHeight="1" thickBot="1">
-      <c r="A35" s="52"/>
-      <c r="B35" s="40"/>
-      <c r="C35" s="57" t="s">
+      <c r="D36" s="71"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="25"/>
+    </row>
+    <row r="37" spans="1:6" ht="20" customHeight="1" thickBot="1">
+      <c r="A37" s="39"/>
+      <c r="B37" s="68"/>
+      <c r="C37" s="77" t="s">
         <v>81</v>
       </c>
-      <c r="D35" s="70"/>
-      <c r="E35" s="71"/>
-      <c r="F35" s="29"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B8:B13"/>
     <mergeCell ref="A2:A13"/>
-    <mergeCell ref="A15:A35"/>
-    <mergeCell ref="B15:B19"/>
-    <mergeCell ref="B21:B35"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B23:B37"/>
+    <mergeCell ref="A15:A37"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:B7"/>
   </mergeCells>

</xml_diff>

<commit_message>
Tuning and setting specification
- Tune solenoids and PID gains
- Modify platformio.ini to accept specific adjustableSettings file
</commit_message>
<xml_diff>
--- a/controller/tuning data/tuning data overview.xlsx
+++ b/controller/tuning data/tuning data overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cfolinus/Documents/MIT/CMF FIDL/07 Control/soft-actuator-controller/controller/tuning data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABACB3D-81B3-0544-8408-109F165D36AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDABEEE-CDF4-3E44-B141-A296CF59AAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="26360" windowHeight="20640" activeTab="1" xr2:uid="{CB76BD02-C45A-F243-9B85-AA0FA8F12FFA}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="32680" windowHeight="20640" xr2:uid="{CB76BD02-C45A-F243-9B85-AA0FA8F12FFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Calibration files" sheetId="1" r:id="rId1"/>
@@ -340,7 +340,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -375,6 +375,11 @@
       <sz val="15"/>
       <color theme="1"/>
       <name val="ArialMT"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="ArialMT"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="24">
@@ -517,7 +522,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -755,21 +760,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -948,7 +938,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1002,18 +992,18 @@
     <xf numFmtId="9" fontId="1" fillId="17" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
@@ -1044,10 +1034,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="20" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1059,12 +1049,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1077,22 +1067,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1112,16 +1099,16 @@
     <xf numFmtId="0" fontId="1" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1129,7 +1116,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="23" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1556,7 +1545,7 @@
       <c r="J2" s="4">
         <v>166</v>
       </c>
-      <c r="K2" s="19">
+      <c r="K2" s="18">
         <v>185</v>
       </c>
       <c r="L2" s="4"/>
@@ -1619,16 +1608,16 @@
       <c r="G4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="18">
+      <c r="H4" s="79">
         <v>0.06</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="79">
         <v>30.9</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="78">
         <v>151</v>
       </c>
-      <c r="K4" s="18">
+      <c r="K4" s="79">
         <v>183</v>
       </c>
       <c r="L4" s="4"/>
@@ -1655,16 +1644,16 @@
       <c r="G5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="19">
         <v>16.899999999999999</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="19">
         <v>8.61</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="19">
         <v>165</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="19">
         <v>171</v>
       </c>
       <c r="L5" s="4"/>
@@ -1691,16 +1680,16 @@
       <c r="G6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="19">
         <v>22.1</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="19">
         <v>11.6</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="19">
         <v>163</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="19">
         <v>170</v>
       </c>
       <c r="L6" s="4"/>
@@ -1724,10 +1713,10 @@
       <c r="G7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
       <c r="L7" s="4"/>
     </row>
     <row r="8" spans="1:12">
@@ -1752,16 +1741,16 @@
       <c r="G8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="19">
         <v>31.4</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="19">
         <v>14.7</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="19">
         <v>155</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="19">
         <v>168</v>
       </c>
       <c r="L8" s="4"/>
@@ -1788,16 +1777,16 @@
       <c r="G9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="19">
         <v>0.06</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="19">
         <v>17.399999999999999</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="19">
         <v>156</v>
       </c>
-      <c r="K9" s="19">
+      <c r="K9" s="18">
         <v>160</v>
       </c>
       <c r="L9" s="4"/>
@@ -1824,16 +1813,16 @@
       <c r="G10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="19">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="19">
         <v>22.7</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="19">
         <v>152</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="19">
         <v>159</v>
       </c>
       <c r="L10" s="4"/>
@@ -1860,16 +1849,16 @@
       <c r="G11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="19">
         <v>0.06</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="19">
         <v>31.4</v>
       </c>
       <c r="J11" s="18">
         <v>145</v>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="19">
         <v>158</v>
       </c>
       <c r="L11" s="4"/>
@@ -2292,10 +2281,10 @@
       <c r="G23" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="19">
         <v>-0.122</v>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="19">
         <v>27.7</v>
       </c>
       <c r="J23" s="18">
@@ -2445,7 +2434,7 @@
       <c r="J27" s="4">
         <v>148</v>
       </c>
-      <c r="K27" s="4">
+      <c r="K27" s="18">
         <v>175</v>
       </c>
       <c r="L27" s="4"/>
@@ -2508,16 +2497,16 @@
       <c r="G29" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H29" s="18">
+      <c r="H29" s="19">
         <v>-0.122</v>
       </c>
-      <c r="I29" s="18">
+      <c r="I29" s="19">
         <v>27.5</v>
       </c>
       <c r="J29" s="18">
         <v>143</v>
       </c>
-      <c r="K29" s="18">
+      <c r="K29" s="19">
         <v>169</v>
       </c>
       <c r="L29" s="4"/>
@@ -2773,10 +2762,10 @@
         <v>63</v>
       </c>
       <c r="C1" s="34"/>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="59" t="s">
+      <c r="E1" s="58" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2809,6 +2798,9 @@
       <c r="E3" s="53">
         <v>-0.122</v>
       </c>
+      <c r="F3">
+        <v>-0.4</v>
+      </c>
     </row>
     <row r="4" spans="1:6" ht="20" customHeight="1">
       <c r="A4" s="47"/>
@@ -2848,6 +2840,9 @@
       <c r="E6" s="53">
         <v>0.11</v>
       </c>
+      <c r="F6">
+        <v>-0.23200000000000001</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="20" customHeight="1">
       <c r="A7" s="47"/>
@@ -2863,6 +2858,10 @@
         <f>E3-E6</f>
         <v>-0.23199999999999998</v>
       </c>
+      <c r="F7" s="53">
+        <f>F3-F6</f>
+        <v>-0.16800000000000001</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="20" customHeight="1">
       <c r="A8" s="47"/>
@@ -2938,25 +2937,25 @@
         <v>65</v>
       </c>
       <c r="D13" s="56">
-        <f>D9-D12</f>
-        <v>-0.05</v>
-      </c>
-      <c r="E13" s="57">
-        <f>E9-E12</f>
-        <v>-0.23199999999999998</v>
+        <f>D12-D9</f>
+        <v>0.05</v>
+      </c>
+      <c r="E13" s="56">
+        <f>E12-E9</f>
+        <v>0.23199999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="20" customHeight="1" thickBot="1">
       <c r="A14" s="49"/>
       <c r="B14" s="42"/>
       <c r="C14" s="24"/>
-      <c r="D14" s="60" t="s">
+      <c r="D14" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="E14" s="61" t="s">
-        <v>1</v>
-      </c>
-      <c r="F14" s="78" t="s">
+      <c r="E14" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="F14" s="77" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2964,35 +2963,35 @@
       <c r="A15" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="64"/>
-      <c r="C15" s="66" t="s">
+      <c r="B15" s="63"/>
+      <c r="C15" s="65" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="69" t="s">
+      <c r="D15" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="65" t="s">
+      <c r="E15" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="F15" s="66"/>
+      <c r="F15" s="65"/>
     </row>
     <row r="16" spans="1:6" ht="20" customHeight="1">
       <c r="A16" s="38"/>
       <c r="B16" s="21"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="67"/>
+      <c r="C16" s="72"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="61"/>
+      <c r="F16" s="66"/>
     </row>
     <row r="17" spans="1:6" ht="20" customHeight="1">
       <c r="A17" s="38"/>
       <c r="B17" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="74" t="s">
+      <c r="C17" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="71">
+      <c r="D17" s="70">
         <f>D4</f>
         <v>151</v>
       </c>
@@ -3005,10 +3004,10 @@
     <row r="18" spans="1:6" ht="20" customHeight="1">
       <c r="A18" s="38"/>
       <c r="B18" s="43"/>
-      <c r="C18" s="74" t="s">
+      <c r="C18" s="73" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="71">
+      <c r="D18" s="70">
         <f>D5</f>
         <v>183</v>
       </c>
@@ -3021,10 +3020,10 @@
     <row r="19" spans="1:6" ht="20" customHeight="1">
       <c r="A19" s="38"/>
       <c r="B19" s="43"/>
-      <c r="C19" s="74" t="s">
+      <c r="C19" s="73" t="s">
         <v>69</v>
       </c>
-      <c r="D19" s="71">
+      <c r="D19" s="70">
         <f>D10</f>
         <v>145</v>
       </c>
@@ -3037,10 +3036,10 @@
     <row r="20" spans="1:6" ht="20" customHeight="1">
       <c r="A20" s="38"/>
       <c r="B20" s="43"/>
-      <c r="C20" s="74" t="s">
+      <c r="C20" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="D20" s="71">
+      <c r="D20" s="70">
         <f>D11</f>
         <v>158</v>
       </c>
@@ -3053,36 +3052,35 @@
     <row r="21" spans="1:6" ht="20" customHeight="1">
       <c r="A21" s="38"/>
       <c r="B21" s="43"/>
-      <c r="C21" s="74" t="s">
+      <c r="C21" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="71">
+      <c r="D21" s="70">
         <f>D7</f>
         <v>-0.05</v>
       </c>
       <c r="E21" s="40">
-        <f>E7</f>
-        <v>-0.23199999999999998</v>
+        <v>0.24</v>
       </c>
       <c r="F21" s="25"/>
     </row>
     <row r="22" spans="1:6" ht="20" customHeight="1">
       <c r="A22" s="38"/>
       <c r="B22" s="20"/>
-      <c r="C22" s="75"/>
-      <c r="D22" s="71"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="70"/>
       <c r="E22" s="40"/>
       <c r="F22" s="25"/>
     </row>
     <row r="23" spans="1:6" ht="20" customHeight="1">
       <c r="A23" s="38"/>
-      <c r="B23" s="63" t="s">
+      <c r="B23" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="C23" s="76" t="s">
+      <c r="C23" s="75" t="s">
         <v>71</v>
       </c>
-      <c r="D23" s="71"/>
+      <c r="D23" s="70"/>
       <c r="E23" s="40"/>
       <c r="F23" s="25" t="s">
         <v>82</v>
@@ -3090,11 +3088,11 @@
     </row>
     <row r="24" spans="1:6" ht="20" customHeight="1">
       <c r="A24" s="38"/>
-      <c r="B24" s="63"/>
-      <c r="C24" s="76" t="s">
+      <c r="B24" s="62"/>
+      <c r="C24" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="71">
+      <c r="D24" s="70">
         <v>0</v>
       </c>
       <c r="E24" s="40">
@@ -3104,19 +3102,19 @@
     </row>
     <row r="25" spans="1:6" ht="20" customHeight="1">
       <c r="A25" s="38"/>
-      <c r="B25" s="63"/>
-      <c r="C25" s="75"/>
-      <c r="D25" s="71"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="70"/>
       <c r="E25" s="40"/>
       <c r="F25" s="25"/>
     </row>
     <row r="26" spans="1:6" ht="20" customHeight="1">
       <c r="A26" s="38"/>
-      <c r="B26" s="63"/>
-      <c r="C26" s="76" t="s">
+      <c r="B26" s="62"/>
+      <c r="C26" s="75" t="s">
         <v>74</v>
       </c>
-      <c r="D26" s="71">
+      <c r="D26" s="70">
         <v>30</v>
       </c>
       <c r="E26" s="40">
@@ -3128,11 +3126,11 @@
     </row>
     <row r="27" spans="1:6" ht="20" customHeight="1">
       <c r="A27" s="38"/>
-      <c r="B27" s="63"/>
-      <c r="C27" s="76" t="s">
+      <c r="B27" s="62"/>
+      <c r="C27" s="75" t="s">
         <v>75</v>
       </c>
-      <c r="D27" s="71">
+      <c r="D27" s="70">
         <v>30</v>
       </c>
       <c r="E27" s="40">
@@ -3144,11 +3142,11 @@
     </row>
     <row r="28" spans="1:6" ht="20" customHeight="1">
       <c r="A28" s="38"/>
-      <c r="B28" s="63"/>
-      <c r="C28" s="76" t="s">
+      <c r="B28" s="62"/>
+      <c r="C28" s="75" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="71">
+      <c r="D28" s="70">
         <v>30</v>
       </c>
       <c r="E28" s="40">
@@ -3160,29 +3158,29 @@
     </row>
     <row r="29" spans="1:6" ht="20" customHeight="1">
       <c r="A29" s="38"/>
-      <c r="B29" s="63"/>
-      <c r="C29" s="75"/>
-      <c r="D29" s="71"/>
+      <c r="B29" s="62"/>
+      <c r="C29" s="74"/>
+      <c r="D29" s="70"/>
       <c r="E29" s="40"/>
       <c r="F29" s="25"/>
     </row>
     <row r="30" spans="1:6" ht="20" customHeight="1">
       <c r="A30" s="38"/>
-      <c r="B30" s="63"/>
-      <c r="C30" s="76" t="s">
+      <c r="B30" s="62"/>
+      <c r="C30" s="75" t="s">
         <v>89</v>
       </c>
-      <c r="D30" s="71"/>
+      <c r="D30" s="70"/>
       <c r="E30" s="40"/>
       <c r="F30" s="25"/>
     </row>
     <row r="31" spans="1:6" ht="20" customHeight="1">
       <c r="A31" s="38"/>
-      <c r="B31" s="63"/>
-      <c r="C31" s="76" t="s">
+      <c r="B31" s="62"/>
+      <c r="C31" s="75" t="s">
         <v>84</v>
       </c>
-      <c r="D31" s="71"/>
+      <c r="D31" s="70"/>
       <c r="E31" s="40"/>
       <c r="F31" s="25" t="s">
         <v>85</v>
@@ -3190,59 +3188,59 @@
     </row>
     <row r="32" spans="1:6" ht="20" customHeight="1">
       <c r="A32" s="38"/>
-      <c r="B32" s="63"/>
-      <c r="C32" s="76" t="s">
+      <c r="B32" s="62"/>
+      <c r="C32" s="75" t="s">
         <v>77</v>
       </c>
-      <c r="D32" s="71"/>
+      <c r="D32" s="70"/>
       <c r="E32" s="40"/>
       <c r="F32" s="25"/>
     </row>
     <row r="33" spans="1:6" ht="20" customHeight="1">
       <c r="A33" s="38"/>
-      <c r="B33" s="63"/>
-      <c r="C33" s="76" t="s">
+      <c r="B33" s="62"/>
+      <c r="C33" s="75" t="s">
         <v>78</v>
       </c>
-      <c r="D33" s="71"/>
+      <c r="D33" s="70"/>
       <c r="E33" s="40"/>
       <c r="F33" s="25"/>
     </row>
     <row r="34" spans="1:6" ht="20" customHeight="1">
       <c r="A34" s="38"/>
-      <c r="B34" s="63"/>
-      <c r="C34" s="76" t="s">
+      <c r="B34" s="62"/>
+      <c r="C34" s="75" t="s">
         <v>79</v>
       </c>
-      <c r="D34" s="71"/>
+      <c r="D34" s="70"/>
       <c r="E34" s="40"/>
       <c r="F34" s="25"/>
     </row>
     <row r="35" spans="1:6" ht="20" customHeight="1">
       <c r="A35" s="38"/>
-      <c r="B35" s="63"/>
-      <c r="C35" s="75"/>
-      <c r="D35" s="71"/>
+      <c r="B35" s="62"/>
+      <c r="C35" s="74"/>
+      <c r="D35" s="70"/>
       <c r="E35" s="40"/>
       <c r="F35" s="25"/>
     </row>
     <row r="36" spans="1:6" ht="20" customHeight="1">
       <c r="A36" s="38"/>
-      <c r="B36" s="63"/>
-      <c r="C36" s="76" t="s">
+      <c r="B36" s="62"/>
+      <c r="C36" s="75" t="s">
         <v>80</v>
       </c>
-      <c r="D36" s="71"/>
+      <c r="D36" s="70"/>
       <c r="E36" s="40"/>
       <c r="F36" s="25"/>
     </row>
     <row r="37" spans="1:6" ht="20" customHeight="1" thickBot="1">
       <c r="A37" s="39"/>
-      <c r="B37" s="68"/>
-      <c r="C37" s="77" t="s">
+      <c r="B37" s="67"/>
+      <c r="C37" s="76" t="s">
         <v>81</v>
       </c>
-      <c r="D37" s="72"/>
+      <c r="D37" s="71"/>
       <c r="E37" s="41"/>
       <c r="F37" s="26"/>
     </row>

</xml_diff>